<commit_message>
SEM Update on Feb 24, 2026
</commit_message>
<xml_diff>
--- a/static/data/source/state_gdp.xlsx
+++ b/static/data/source/state_gdp.xlsx
@@ -1,29 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29816"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aboddupalli\Box\TIS\TPC\CENTER\SLFI\Interactive Data Tools\SEM\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35E1657-AB60-48AB-B62A-A867FAECB657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{E35E1657-AB60-48AB-B62A-A867FAECB657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{868C494D-D4B0-4597-838E-A53B40BD3726}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TABLE_1" sheetId="4" r:id="rId1"/>
     <sheet name="TABLE_2" sheetId="5" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +39,259 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="138">
   <si>
+    <t>State Gross Domestic Product (GDP); Millions of Real Dollars</t>
+  </si>
+  <si>
     <t>Geography</t>
+  </si>
+  <si>
+    <t>2005 Q1</t>
+  </si>
+  <si>
+    <t>2005 Q2</t>
+  </si>
+  <si>
+    <t>2005 Q3</t>
+  </si>
+  <si>
+    <t>2005 Q4</t>
+  </si>
+  <si>
+    <t>2006 Q1</t>
+  </si>
+  <si>
+    <t>2006 Q2</t>
+  </si>
+  <si>
+    <t>2006 Q3</t>
+  </si>
+  <si>
+    <t>2006 Q4</t>
+  </si>
+  <si>
+    <t>2007 Q1</t>
+  </si>
+  <si>
+    <t>2007 Q2</t>
+  </si>
+  <si>
+    <t>2007 Q3</t>
+  </si>
+  <si>
+    <t>2007 Q4</t>
+  </si>
+  <si>
+    <t>2008 Q1</t>
+  </si>
+  <si>
+    <t>2008 Q2</t>
+  </si>
+  <si>
+    <t>2008 Q3</t>
+  </si>
+  <si>
+    <t>2008 Q4</t>
+  </si>
+  <si>
+    <t>2009 Q1</t>
+  </si>
+  <si>
+    <t>2009 Q2</t>
+  </si>
+  <si>
+    <t>2009 Q3</t>
+  </si>
+  <si>
+    <t>2009 Q4</t>
+  </si>
+  <si>
+    <t>2010 Q1</t>
+  </si>
+  <si>
+    <t>2010 Q2</t>
+  </si>
+  <si>
+    <t>2010 Q3</t>
+  </si>
+  <si>
+    <t>2010 Q4</t>
+  </si>
+  <si>
+    <t>2011 Q1</t>
+  </si>
+  <si>
+    <t>2011 Q2</t>
+  </si>
+  <si>
+    <t>2011 Q3</t>
+  </si>
+  <si>
+    <t>2011 Q4</t>
+  </si>
+  <si>
+    <t>2012 Q1</t>
+  </si>
+  <si>
+    <t>2012 Q2</t>
+  </si>
+  <si>
+    <t>2012 Q3</t>
+  </si>
+  <si>
+    <t>2012 Q4</t>
+  </si>
+  <si>
+    <t>2013 Q1</t>
+  </si>
+  <si>
+    <t>2013 Q2</t>
+  </si>
+  <si>
+    <t>2013 Q3</t>
+  </si>
+  <si>
+    <t>2013 Q4</t>
+  </si>
+  <si>
+    <t>2014 Q1</t>
+  </si>
+  <si>
+    <t>2014 Q2</t>
+  </si>
+  <si>
+    <t>2014 Q3</t>
+  </si>
+  <si>
+    <t>2014 Q4</t>
+  </si>
+  <si>
+    <t>2015 Q1</t>
+  </si>
+  <si>
+    <t>2015 Q2</t>
+  </si>
+  <si>
+    <t>2015 Q3</t>
+  </si>
+  <si>
+    <t>2015 Q4</t>
+  </si>
+  <si>
+    <t>2016 Q1</t>
+  </si>
+  <si>
+    <t>2016 Q2</t>
+  </si>
+  <si>
+    <t>2016 Q3</t>
+  </si>
+  <si>
+    <t>2016 Q4</t>
+  </si>
+  <si>
+    <t>2017 Q1</t>
+  </si>
+  <si>
+    <t>2017 Q2</t>
+  </si>
+  <si>
+    <t>2017 Q3</t>
+  </si>
+  <si>
+    <t>2017 Q4</t>
+  </si>
+  <si>
+    <t>2018 Q1</t>
+  </si>
+  <si>
+    <t>2018 Q2</t>
+  </si>
+  <si>
+    <t>2018 Q3</t>
+  </si>
+  <si>
+    <t>2018 Q4</t>
+  </si>
+  <si>
+    <t>2019 Q1</t>
+  </si>
+  <si>
+    <t>2019 Q2</t>
+  </si>
+  <si>
+    <t>2019 Q3</t>
+  </si>
+  <si>
+    <t>2019 Q4</t>
+  </si>
+  <si>
+    <t>2020 Q1</t>
+  </si>
+  <si>
+    <t>2020 Q2</t>
+  </si>
+  <si>
+    <t>2020 Q3</t>
+  </si>
+  <si>
+    <t>2020 Q4</t>
+  </si>
+  <si>
+    <t>2021 Q1</t>
+  </si>
+  <si>
+    <t>2021 Q2</t>
+  </si>
+  <si>
+    <t>2021 Q3</t>
+  </si>
+  <si>
+    <t>2021 Q4</t>
+  </si>
+  <si>
+    <t>2022 Q1</t>
+  </si>
+  <si>
+    <t>2022 Q2</t>
+  </si>
+  <si>
+    <t>2022 Q3</t>
+  </si>
+  <si>
+    <t>2022 Q4</t>
+  </si>
+  <si>
+    <t>2023 Q1</t>
+  </si>
+  <si>
+    <t>2023 Q2</t>
+  </si>
+  <si>
+    <t>2023 Q3</t>
+  </si>
+  <si>
+    <t>2023 Q4</t>
+  </si>
+  <si>
+    <t>2024 Q1</t>
+  </si>
+  <si>
+    <t>2024 Q2</t>
+  </si>
+  <si>
+    <t>2024 Q3</t>
+  </si>
+  <si>
+    <t>2024 Q4</t>
+  </si>
+  <si>
+    <t>2025 Q1</t>
+  </si>
+  <si>
+    <t>2025 Q2</t>
+  </si>
+  <si>
+    <t>2025 Q3</t>
   </si>
   <si>
     <t>United States</t>
@@ -192,259 +450,7 @@
     <t>Wyoming</t>
   </si>
   <si>
-    <t>2018 Q1</t>
-  </si>
-  <si>
-    <t>2018 Q2</t>
-  </si>
-  <si>
-    <t>2018 Q3</t>
-  </si>
-  <si>
-    <t>2018 Q4</t>
-  </si>
-  <si>
-    <t>2019 Q1</t>
-  </si>
-  <si>
-    <t>State Gross Domestic Product (GDP); Millions of Real Dollars</t>
-  </si>
-  <si>
     <t>State Gross Domestic Product (GDP); Year-over-year</t>
-  </si>
-  <si>
-    <t>2019 Q2</t>
-  </si>
-  <si>
-    <t>2019 Q3</t>
-  </si>
-  <si>
-    <t>2019 Q4</t>
-  </si>
-  <si>
-    <t>2020 Q1</t>
-  </si>
-  <si>
-    <t>2020 Q2</t>
-  </si>
-  <si>
-    <t>2020 Q3</t>
-  </si>
-  <si>
-    <t>2020 Q4</t>
-  </si>
-  <si>
-    <t>2021 Q1</t>
-  </si>
-  <si>
-    <t>2021 Q2</t>
-  </si>
-  <si>
-    <t>2021 Q3</t>
-  </si>
-  <si>
-    <t>2021 Q4</t>
-  </si>
-  <si>
-    <t>2022 Q1</t>
-  </si>
-  <si>
-    <t>2022 Q2</t>
-  </si>
-  <si>
-    <t>2022 Q3</t>
-  </si>
-  <si>
-    <t>2022 Q4</t>
-  </si>
-  <si>
-    <t>2023 Q1</t>
-  </si>
-  <si>
-    <t>2023 Q2</t>
-  </si>
-  <si>
-    <t>2023 Q3</t>
-  </si>
-  <si>
-    <t>2023 Q4</t>
-  </si>
-  <si>
-    <t>2024 Q1</t>
-  </si>
-  <si>
-    <t>2024 Q2</t>
-  </si>
-  <si>
-    <t>2005 Q1</t>
-  </si>
-  <si>
-    <t>2005 Q2</t>
-  </si>
-  <si>
-    <t>2005 Q3</t>
-  </si>
-  <si>
-    <t>2005 Q4</t>
-  </si>
-  <si>
-    <t>2006 Q1</t>
-  </si>
-  <si>
-    <t>2006 Q2</t>
-  </si>
-  <si>
-    <t>2006 Q3</t>
-  </si>
-  <si>
-    <t>2006 Q4</t>
-  </si>
-  <si>
-    <t>2007 Q1</t>
-  </si>
-  <si>
-    <t>2007 Q2</t>
-  </si>
-  <si>
-    <t>2007 Q3</t>
-  </si>
-  <si>
-    <t>2007 Q4</t>
-  </si>
-  <si>
-    <t>2008 Q1</t>
-  </si>
-  <si>
-    <t>2008 Q2</t>
-  </si>
-  <si>
-    <t>2008 Q3</t>
-  </si>
-  <si>
-    <t>2008 Q4</t>
-  </si>
-  <si>
-    <t>2009 Q1</t>
-  </si>
-  <si>
-    <t>2009 Q2</t>
-  </si>
-  <si>
-    <t>2009 Q3</t>
-  </si>
-  <si>
-    <t>2009 Q4</t>
-  </si>
-  <si>
-    <t>2010 Q1</t>
-  </si>
-  <si>
-    <t>2010 Q2</t>
-  </si>
-  <si>
-    <t>2010 Q3</t>
-  </si>
-  <si>
-    <t>2010 Q4</t>
-  </si>
-  <si>
-    <t>2011 Q1</t>
-  </si>
-  <si>
-    <t>2011 Q2</t>
-  </si>
-  <si>
-    <t>2011 Q3</t>
-  </si>
-  <si>
-    <t>2011 Q4</t>
-  </si>
-  <si>
-    <t>2012 Q1</t>
-  </si>
-  <si>
-    <t>2012 Q2</t>
-  </si>
-  <si>
-    <t>2012 Q3</t>
-  </si>
-  <si>
-    <t>2012 Q4</t>
-  </si>
-  <si>
-    <t>2013 Q1</t>
-  </si>
-  <si>
-    <t>2013 Q2</t>
-  </si>
-  <si>
-    <t>2013 Q3</t>
-  </si>
-  <si>
-    <t>2013 Q4</t>
-  </si>
-  <si>
-    <t>2014 Q1</t>
-  </si>
-  <si>
-    <t>2014 Q2</t>
-  </si>
-  <si>
-    <t>2014 Q3</t>
-  </si>
-  <si>
-    <t>2014 Q4</t>
-  </si>
-  <si>
-    <t>2015 Q1</t>
-  </si>
-  <si>
-    <t>2015 Q2</t>
-  </si>
-  <si>
-    <t>2015 Q3</t>
-  </si>
-  <si>
-    <t>2015 Q4</t>
-  </si>
-  <si>
-    <t>2016 Q1</t>
-  </si>
-  <si>
-    <t>2016 Q2</t>
-  </si>
-  <si>
-    <t>2016 Q3</t>
-  </si>
-  <si>
-    <t>2016 Q4</t>
-  </si>
-  <si>
-    <t>2017 Q1</t>
-  </si>
-  <si>
-    <t>2017 Q2</t>
-  </si>
-  <si>
-    <t>2017 Q3</t>
-  </si>
-  <si>
-    <t>2017 Q4</t>
-  </si>
-  <si>
-    <t>2024 Q3</t>
-  </si>
-  <si>
-    <t>2024 Q4</t>
-  </si>
-  <si>
-    <t>2025 Q1</t>
-  </si>
-  <si>
-    <t>2025 Q2</t>
-  </si>
-  <si>
-    <t>2025 Q3</t>
   </si>
 </sst>
 </file>
@@ -454,7 +460,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -540,7 +546,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -568,6 +574,7 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,9 +594,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -627,7 +634,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -733,7 +740,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -875,7 +882,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -883,293 +890,296 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CF56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:CG56"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="18.109375" style="2" customWidth="1"/>
-    <col min="2" max="24" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" style="2" customWidth="1"/>
+    <col min="2" max="24" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="30" max="31" width="14" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="14" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="14" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="14" bestFit="1" customWidth="1"/>
-    <col min="40" max="46" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="46" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="14" bestFit="1" customWidth="1"/>
-    <col min="48" max="60" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="48" max="60" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="14" bestFit="1" customWidth="1"/>
-    <col min="62" max="65" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="62" max="65" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="66" max="66" width="14" bestFit="1" customWidth="1"/>
-    <col min="67" max="78" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="79" max="84" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="78" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="79" max="84" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:85">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:85" ht="15"/>
+    <row r="4" spans="1:85" ht="15">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="P4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="R4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="U4" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="V4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="W4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="X4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z4" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA4" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB4" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD4" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF4" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH4" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ4" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK4" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AM4" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AN4" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="AO4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="AP4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AQ4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AR4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AS4" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="AT4" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="AU4" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV4" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AW4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="AX4" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AY4" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AZ4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="BA4" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="BB4" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="BC4" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="BD4" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="BE4" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="BF4" s="8" t="s">
         <v>58</v>
       </c>
+      <c r="BG4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="BH4" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="BI4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="BJ4" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="BK4" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="BL4" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="BM4" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="BN4" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="BO4" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="BP4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="BQ4" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="BR4" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="BS4" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="BT4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="BU4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="BV4" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="BW4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="BX4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="BY4" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="BZ4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="CA4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="CB4" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="CC4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="CD4" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="CE4" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="CF4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="CG4" s="8"/>
     </row>
-    <row r="4" spans="1:84" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F4" s="8" t="s">
+    <row r="5" spans="1:85" ht="15">
+      <c r="A5" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="K4" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="L4" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="M4" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="N4" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="O4" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="P4" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q4" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="R4" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="S4" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="T4" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="U4" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="W4" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="X4" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y4" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z4" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA4" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="AB4" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="AC4" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="AD4" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="AE4" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="AF4" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="AG4" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="AH4" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="AI4" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="AJ4" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="AK4" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="AL4" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="AM4" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="AN4" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="AO4" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="AP4" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="AQ4" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="AR4" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="AS4" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="AT4" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="AU4" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="AV4" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="AW4" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="AX4" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="AY4" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="AZ4" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="BA4" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="BB4" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="BC4" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="BD4" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="BE4" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="BF4" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="BG4" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="BH4" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="BI4" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="BJ4" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="BK4" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="BL4" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="BM4" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="BN4" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="BO4" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="BP4" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="BQ4" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="BR4" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="BS4" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="BT4" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="BU4" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="BV4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="BW4" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="BX4" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="BY4" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="BZ4" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="CA4" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="CB4" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="CC4" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="CD4" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="CE4" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="CF4" s="8" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:84" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>1</v>
       </c>
       <c r="B5" s="6">
         <v>20508045.868557665</v>
@@ -1420,10 +1430,11 @@
       <c r="CF5" s="7">
         <v>31098027</v>
       </c>
+      <c r="CG5" s="11"/>
     </row>
-    <row r="6" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:85">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="B6" s="6">
         <v>256996.59501738215</v>
@@ -1674,10 +1685,11 @@
       <c r="CF6" s="7">
         <v>344535.1</v>
       </c>
+      <c r="CG6" s="11"/>
     </row>
-    <row r="7" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:85">
       <c r="A7" s="4" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="B7" s="6">
         <v>57315.332219649979</v>
@@ -1928,10 +1940,11 @@
       <c r="CF7" s="7">
         <v>75289.600000000006</v>
       </c>
+      <c r="CG7" s="11"/>
     </row>
-    <row r="8" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:85">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="B8" s="6">
         <v>366144.6152179279</v>
@@ -2182,10 +2195,11 @@
       <c r="CF8" s="7">
         <v>604334.5</v>
       </c>
+      <c r="CG8" s="11"/>
     </row>
-    <row r="9" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:85">
       <c r="A9" s="4" t="s">
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="B9" s="6">
         <v>147439.10724093963</v>
@@ -2436,10 +2450,11 @@
       <c r="CF9" s="7">
         <v>200475.5</v>
       </c>
+      <c r="CG9" s="11"/>
     </row>
-    <row r="10" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:85">
       <c r="A10" s="4" t="s">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="B10" s="6">
         <v>2531641.4064370617</v>
@@ -2690,10 +2705,11 @@
       <c r="CF10" s="7">
         <v>4296452.0999999996</v>
       </c>
+      <c r="CG10" s="11"/>
     </row>
-    <row r="11" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:85">
       <c r="A11" s="4" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="B11" s="6">
         <v>334722.88434968761</v>
@@ -2944,10 +2960,11 @@
       <c r="CF11" s="7">
         <v>589908.5</v>
       </c>
+      <c r="CG11" s="11"/>
     </row>
-    <row r="12" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:85">
       <c r="A12" s="4" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="B12" s="6">
         <v>330600.46244466671</v>
@@ -3198,10 +3215,11 @@
       <c r="CF12" s="7">
         <v>381516.7</v>
       </c>
+      <c r="CG12" s="11"/>
     </row>
-    <row r="13" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:85">
       <c r="A13" s="4" t="s">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="B13" s="6">
         <v>88691.813003941308</v>
@@ -3452,10 +3470,11 @@
       <c r="CF13" s="7">
         <v>118576.7</v>
       </c>
+      <c r="CG13" s="11"/>
     </row>
-    <row r="14" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:85">
       <c r="A14" s="4" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="B14" s="6">
         <v>143983.86895996192</v>
@@ -3706,10 +3725,11 @@
       <c r="CF14" s="7">
         <v>194298.9</v>
       </c>
+      <c r="CG14" s="11"/>
     </row>
-    <row r="15" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:85">
       <c r="A15" s="4" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="B15" s="6">
         <v>1152503.9681409076</v>
@@ -3960,10 +3980,11 @@
       <c r="CF15" s="7">
         <v>1852346.3</v>
       </c>
+      <c r="CG15" s="11"/>
     </row>
-    <row r="16" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:85">
       <c r="A16" s="4" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="B16" s="6">
         <v>623573.0604405459</v>
@@ -4214,10 +4235,11 @@
       <c r="CF16" s="7">
         <v>935786.8</v>
       </c>
+      <c r="CG16" s="11"/>
     </row>
-    <row r="17" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:85">
       <c r="A17" s="4" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="B17" s="6">
         <v>95426.694709288335</v>
@@ -4468,10 +4490,11 @@
       <c r="CF17" s="7">
         <v>125476.9</v>
       </c>
+      <c r="CG17" s="11"/>
     </row>
-    <row r="18" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:85">
       <c r="A18" s="4" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="B18" s="6">
         <v>78091.732858570016</v>
@@ -4722,10 +4745,11 @@
       <c r="CF18" s="7">
         <v>136846.79999999999</v>
       </c>
+      <c r="CG18" s="11"/>
     </row>
-    <row r="19" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:85">
       <c r="A19" s="4" t="s">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="B19" s="6">
         <v>976485.14796974522</v>
@@ -4976,10 +5000,11 @@
       <c r="CF19" s="7">
         <v>1216429.8</v>
       </c>
+      <c r="CG19" s="11"/>
     </row>
-    <row r="20" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:85">
       <c r="A20" s="4" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="B20" s="6">
         <v>393382.99170542503</v>
@@ -5230,10 +5255,11 @@
       <c r="CF20" s="7">
         <v>551815.6</v>
       </c>
+      <c r="CG20" s="11"/>
     </row>
-    <row r="21" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:85">
       <c r="A21" s="4" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="B21" s="6">
         <v>204157.69531079024</v>
@@ -5484,10 +5510,11 @@
       <c r="CF21" s="7">
         <v>280071.2</v>
       </c>
+      <c r="CG21" s="11"/>
     </row>
-    <row r="22" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:85">
       <c r="A22" s="4" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="B22" s="6">
         <v>169855.56483824845</v>
@@ -5738,10 +5765,11 @@
       <c r="CF22" s="7">
         <v>244987</v>
       </c>
+      <c r="CG22" s="11"/>
     </row>
-    <row r="23" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:85">
       <c r="A23" s="4" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="B23" s="6">
         <v>236601.59705150148</v>
@@ -5992,10 +6020,11 @@
       <c r="CF23" s="7">
         <v>311071.5</v>
       </c>
+      <c r="CG23" s="11"/>
     </row>
-    <row r="24" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:85">
       <c r="A24" s="4" t="s">
-        <v>20</v>
+        <v>104</v>
       </c>
       <c r="B24" s="6">
         <v>328647.12094393926</v>
@@ -6246,10 +6275,11 @@
       <c r="CF24" s="7">
         <v>343643.9</v>
       </c>
+      <c r="CG24" s="11"/>
     </row>
-    <row r="25" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:85">
       <c r="A25" s="4" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="B25" s="6">
         <v>78069.235377014804</v>
@@ -6500,10 +6530,11 @@
       <c r="CF25" s="7">
         <v>103894.6</v>
       </c>
+      <c r="CG25" s="11"/>
     </row>
-    <row r="26" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:85">
       <c r="A26" s="4" t="s">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="B26" s="6">
         <v>417695.6692519667</v>
@@ -6754,10 +6785,11 @@
       <c r="CF26" s="7">
         <v>574376.6</v>
       </c>
+      <c r="CG26" s="11"/>
     </row>
-    <row r="27" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:85">
       <c r="A27" s="4" t="s">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="B27" s="6">
         <v>528519.23853006132</v>
@@ -7008,10 +7040,11 @@
       <c r="CF27" s="7">
         <v>828256.7</v>
       </c>
+      <c r="CG27" s="11"/>
     </row>
-    <row r="28" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:85">
       <c r="A28" s="4" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="B28" s="6">
         <v>638056.72335325123</v>
@@ -7262,10 +7295,11 @@
       <c r="CF28" s="7">
         <v>738308</v>
       </c>
+      <c r="CG28" s="11"/>
     </row>
-    <row r="29" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:85">
       <c r="A29" s="4" t="s">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="B29" s="6">
         <v>393833.03252400563</v>
@@ -7516,10 +7550,11 @@
       <c r="CF29" s="7">
         <v>535819.1</v>
       </c>
+      <c r="CG29" s="11"/>
     </row>
-    <row r="30" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:85">
       <c r="A30" s="4" t="s">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="B30" s="6">
         <v>135588.94804195804</v>
@@ -7770,10 +7805,11 @@
       <c r="CF30" s="7">
         <v>166735.20000000001</v>
       </c>
+      <c r="CG30" s="11"/>
     </row>
-    <row r="31" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:85">
       <c r="A31" s="4" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="B31" s="6">
         <v>372181.51686500397</v>
@@ -8024,10 +8060,11 @@
       <c r="CF31" s="7">
         <v>473652.1</v>
       </c>
+      <c r="CG31" s="11"/>
     </row>
-    <row r="32" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:85">
       <c r="A32" s="4" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="B32" s="6">
         <v>51741.954856947588</v>
@@ -8278,10 +8315,11 @@
       <c r="CF32" s="7">
         <v>83185.600000000006</v>
       </c>
+      <c r="CG32" s="11"/>
     </row>
-    <row r="33" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:85">
       <c r="A33" s="4" t="s">
-        <v>29</v>
+        <v>113</v>
       </c>
       <c r="B33" s="6">
         <v>122704.6717020723</v>
@@ -8532,10 +8570,11 @@
       <c r="CF33" s="7">
         <v>200484.7</v>
       </c>
+      <c r="CG33" s="11"/>
     </row>
-    <row r="34" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:85">
       <c r="A34" s="4" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="B34" s="6">
         <v>197187.06613498068</v>
@@ -8786,10 +8825,11 @@
       <c r="CF34" s="7">
         <v>284135.90000000002</v>
       </c>
+      <c r="CG34" s="11"/>
     </row>
-    <row r="35" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:85">
       <c r="A35" s="4" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="B35" s="6">
         <v>89675.558940535135</v>
@@ -9040,10 +9080,11 @@
       <c r="CF35" s="7">
         <v>126921.1</v>
       </c>
+      <c r="CG35" s="11"/>
     </row>
-    <row r="36" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:85">
       <c r="A36" s="4" t="s">
-        <v>32</v>
+        <v>116</v>
       </c>
       <c r="B36" s="6">
         <v>700849.97635980579</v>
@@ -9294,10 +9335,11 @@
       <c r="CF36" s="7">
         <v>896408.1</v>
       </c>
+      <c r="CG36" s="11"/>
     </row>
-    <row r="37" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:85">
       <c r="A37" s="4" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="B37" s="6">
         <v>109501.301009128</v>
@@ -9548,10 +9590,11 @@
       <c r="CF37" s="7">
         <v>153972.29999999999</v>
       </c>
+      <c r="CG37" s="11"/>
     </row>
-    <row r="38" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:85">
       <c r="A38" s="4" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="B38" s="6">
         <v>1670229.3207352478</v>
@@ -9802,10 +9845,11 @@
       <c r="CF38" s="7">
         <v>2496819.7999999998</v>
       </c>
+      <c r="CG38" s="11"/>
     </row>
-    <row r="39" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:85">
       <c r="A39" s="4" t="s">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="B39" s="6">
         <v>579836.2570229742</v>
@@ -10056,10 +10100,11 @@
       <c r="CF39" s="7">
         <v>905215</v>
       </c>
+      <c r="CG39" s="11"/>
     </row>
-    <row r="40" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:85">
       <c r="A40" s="4" t="s">
-        <v>36</v>
+        <v>120</v>
       </c>
       <c r="B40" s="6">
         <v>38106.658967533564</v>
@@ -10310,10 +10355,11 @@
       <c r="CF40" s="7">
         <v>81926.3</v>
       </c>
+      <c r="CG40" s="11"/>
     </row>
-    <row r="41" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:85">
       <c r="A41" s="4" t="s">
-        <v>37</v>
+        <v>121</v>
       </c>
       <c r="B41" s="6">
         <v>767527.81150919478</v>
@@ -10564,10 +10610,11 @@
       <c r="CF41" s="7">
         <v>979083</v>
       </c>
+      <c r="CG41" s="11"/>
     </row>
-    <row r="42" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:85">
       <c r="A42" s="4" t="s">
-        <v>38</v>
+        <v>122</v>
       </c>
       <c r="B42" s="6">
         <v>180128.1573984526</v>
@@ -10818,10 +10865,11 @@
       <c r="CF42" s="7">
         <v>276723</v>
       </c>
+      <c r="CG42" s="11"/>
     </row>
-    <row r="43" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:85">
       <c r="A43" s="4" t="s">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="B43" s="6">
         <v>215847.11985183935</v>
@@ -11072,10 +11120,11 @@
       <c r="CF43" s="7">
         <v>346483.6</v>
       </c>
+      <c r="CG43" s="11"/>
     </row>
-    <row r="44" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:85">
       <c r="A44" s="4" t="s">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="B44" s="6">
         <v>803468.82792186446</v>
@@ -11326,10 +11375,11 @@
       <c r="CF44" s="7">
         <v>1069852.3</v>
       </c>
+      <c r="CG44" s="11"/>
     </row>
-    <row r="45" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:85">
       <c r="A45" s="4" t="s">
-        <v>41</v>
+        <v>125</v>
       </c>
       <c r="B45" s="6">
         <v>72239.183694276799</v>
@@ -11580,10 +11630,11 @@
       <c r="CF45" s="7">
         <v>84799.6</v>
       </c>
+      <c r="CG45" s="11"/>
     </row>
-    <row r="46" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:85">
       <c r="A46" s="4" t="s">
-        <v>42</v>
+        <v>126</v>
       </c>
       <c r="B46" s="6">
         <v>241616.01013916035</v>
@@ -11834,10 +11885,11 @@
       <c r="CF46" s="7">
         <v>383139.5</v>
       </c>
+      <c r="CG46" s="11"/>
     </row>
-    <row r="47" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:85">
       <c r="A47" s="4" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="B47" s="6">
         <v>54447.755530880604</v>
@@ -12088,10 +12140,11 @@
       <c r="CF47" s="7">
         <v>81595.3</v>
       </c>
+      <c r="CG47" s="11"/>
     </row>
-    <row r="48" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:85">
       <c r="A48" s="4" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="B48" s="6">
         <v>377203.82288590021</v>
@@ -12342,10 +12395,11 @@
       <c r="CF48" s="7">
         <v>596585.6</v>
       </c>
+      <c r="CG48" s="11"/>
     </row>
-    <row r="49" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:85">
       <c r="A49" s="4" t="s">
-        <v>45</v>
+        <v>129</v>
       </c>
       <c r="B49" s="6">
         <v>1464571.8060863942</v>
@@ -12596,10 +12650,11 @@
       <c r="CF49" s="7">
         <v>2935858.8</v>
       </c>
+      <c r="CG49" s="11"/>
     </row>
-    <row r="50" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:85">
       <c r="A50" s="4" t="s">
-        <v>46</v>
+        <v>130</v>
       </c>
       <c r="B50" s="6">
         <v>152242.22688827972</v>
@@ -12850,10 +12905,11 @@
       <c r="CF50" s="7">
         <v>319043.7</v>
       </c>
+      <c r="CG50" s="11"/>
     </row>
-    <row r="51" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:85">
       <c r="A51" s="4" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="B51" s="6">
         <v>38427.755858382261</v>
@@ -13104,10 +13160,11 @@
       <c r="CF51" s="7">
         <v>48887.8</v>
       </c>
+      <c r="CG51" s="11"/>
     </row>
-    <row r="52" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:85">
       <c r="A52" s="4" t="s">
-        <v>48</v>
+        <v>132</v>
       </c>
       <c r="B52" s="6">
         <v>559524.28233124921</v>
@@ -13358,10 +13415,11 @@
       <c r="CF52" s="7">
         <v>807318.9</v>
       </c>
+      <c r="CG52" s="11"/>
     </row>
-    <row r="53" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:85">
       <c r="A53" s="4" t="s">
-        <v>49</v>
+        <v>133</v>
       </c>
       <c r="B53" s="6">
         <v>442546.83666836988</v>
@@ -13612,10 +13670,11 @@
       <c r="CF53" s="7">
         <v>903683.2</v>
       </c>
+      <c r="CG53" s="11"/>
     </row>
-    <row r="54" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:85">
       <c r="A54" s="4" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="B54" s="6">
         <v>88750.584501088189</v>
@@ -13866,10 +13925,11 @@
       <c r="CF54" s="7">
         <v>110273.3</v>
       </c>
+      <c r="CG54" s="11"/>
     </row>
-    <row r="55" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:85">
       <c r="A55" s="4" t="s">
-        <v>51</v>
+        <v>135</v>
       </c>
       <c r="B55" s="6">
         <v>369732.85993833788</v>
@@ -14120,10 +14180,11 @@
       <c r="CF55" s="7">
         <v>478547.6</v>
       </c>
+      <c r="CG55" s="11"/>
     </row>
-    <row r="56" spans="1:84" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:85">
       <c r="A56" s="4" t="s">
-        <v>52</v>
+        <v>136</v>
       </c>
       <c r="B56" s="6">
         <v>42661.043057190371</v>
@@ -14374,6 +14435,7 @@
       <c r="CF56" s="7">
         <v>52961.3</v>
       </c>
+      <c r="CG56" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -14384,264 +14446,266 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:CB56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:CC56"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="18.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" style="2" customWidth="1"/>
     <col min="2" max="23" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="24" max="80" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:81">
       <c r="A1" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:81" ht="15"/>
+    <row r="4" spans="1:81" ht="24">
+      <c r="A4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="R4" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="T4" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA4" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB4" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC4" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD4" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE4" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF4" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG4" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AH4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI4" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AJ4" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK4" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="AL4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AM4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN4" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="AP4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="AQ4" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AR4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AS4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="AT4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AU4" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AV4" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="AW4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="AY4" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AZ4" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="BA4" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="BB4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="BC4" s="9" t="s">
         <v>59</v>
       </c>
+      <c r="BD4" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="BE4" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="BF4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="BG4" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="BH4" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="BI4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="BJ4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="BK4" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BL4" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="BM4" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="BN4" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="BO4" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="BP4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="BQ4" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="BR4" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS4" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="BT4" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="BU4" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="BV4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="BW4" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="BX4" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="BY4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="BZ4" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="CA4" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="CB4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="CC4" s="8"/>
     </row>
-    <row r="4" spans="1:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="9" t="s">
+    <row r="5" spans="1:81" ht="15">
+      <c r="A5" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="O4" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q4" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="R4" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="S4" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="T4" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="U4" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="V4" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="W4" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="X4" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="Y4" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z4" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="AA4" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="AB4" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="AC4" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="AD4" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="AE4" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="AF4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="AG4" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="AH4" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="AI4" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AJ4" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="AK4" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="AL4" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="AM4" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="AN4" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO4" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="AP4" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="AQ4" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="AR4" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="AS4" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="AT4" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="AU4" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="AV4" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="AW4" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="AX4" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="AY4" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="AZ4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="BA4" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="BB4" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="BC4" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="BD4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="BE4" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="BF4" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="BG4" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="BH4" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="BI4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="BJ4" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="BK4" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="BL4" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="BM4" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="BN4" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="BO4" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="BP4" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="BQ4" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="BR4" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="BS4" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="BT4" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="BU4" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="BV4" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="BW4" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="BX4" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="BY4" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="BZ4" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="CA4" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="CB4" s="8" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:80" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>1</v>
       </c>
       <c r="B5" s="5">
         <v>3.2119914346895144</v>
@@ -14881,9 +14945,9 @@
         <v>2.3347116067326623</v>
       </c>
     </row>
-    <row r="6" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:81">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="B6" s="5">
         <v>1.7734579108178867</v>
@@ -15123,9 +15187,9 @@
         <v>1.7698222614395522</v>
       </c>
     </row>
-    <row r="7" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:81">
       <c r="A7" s="4" t="s">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="B7" s="5">
         <v>4.0713303896166897</v>
@@ -15365,9 +15429,9 @@
         <v>2.4855036015602008</v>
       </c>
     </row>
-    <row r="8" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:81">
       <c r="A8" s="4" t="s">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="B8" s="5">
         <v>5.3870762889562247</v>
@@ -15607,9 +15671,9 @@
         <v>2.1012919053936945</v>
       </c>
     </row>
-    <row r="9" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:81">
       <c r="A9" s="4" t="s">
-        <v>5</v>
+        <v>89</v>
       </c>
       <c r="B9" s="5">
         <v>2.7595327798708582</v>
@@ -15849,9 +15913,9 @@
         <v>2.237858074004746</v>
       </c>
     </row>
-    <row r="10" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:81">
       <c r="A10" s="4" t="s">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="B10" s="5">
         <v>5.0766883700656731</v>
@@ -16091,9 +16155,9 @@
         <v>2.7953103471036074</v>
       </c>
     </row>
-    <row r="11" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:81">
       <c r="A11" s="4" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="B11" s="5">
         <v>2.2449662184761436</v>
@@ -16333,9 +16397,9 @@
         <v>2.2693042249584723</v>
       </c>
     </row>
-    <row r="12" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:81">
       <c r="A12" s="4" t="s">
-        <v>8</v>
+        <v>92</v>
       </c>
       <c r="B12" s="5">
         <v>5.3830780904339974</v>
@@ -16575,9 +16639,9 @@
         <v>2.9881067058341109</v>
       </c>
     </row>
-    <row r="13" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:81">
       <c r="A13" s="4" t="s">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="B13" s="5">
         <v>3.5837856712059173</v>
@@ -16817,9 +16881,9 @@
         <v>2.3076175670423624</v>
       </c>
     </row>
-    <row r="14" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:81">
       <c r="A14" s="4" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="B14" s="5">
         <v>-0.17540392311874145</v>
@@ -17059,9 +17123,9 @@
         <v>1.3564165367772456</v>
       </c>
     </row>
-    <row r="15" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:81">
       <c r="A15" s="4" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="B15" s="5">
         <v>3.4901718900927352</v>
@@ -17301,9 +17365,9 @@
         <v>3.0180741315390907</v>
       </c>
     </row>
-    <row r="16" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:81">
       <c r="A16" s="4" t="s">
-        <v>12</v>
+        <v>96</v>
       </c>
       <c r="B16" s="5">
         <v>1.426474186444836</v>
@@ -17543,9 +17607,9 @@
         <v>2.2659819255010634</v>
       </c>
     </row>
-    <row r="17" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:80">
       <c r="A17" s="4" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="B17" s="5">
         <v>2.8471698572158357</v>
@@ -17785,9 +17849,9 @@
         <v>2.2006692757075563</v>
       </c>
     </row>
-    <row r="18" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:80">
       <c r="A18" s="4" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="B18" s="5">
         <v>4.1615085468482258</v>
@@ -18027,9 +18091,9 @@
         <v>1.6133125475836612</v>
       </c>
     </row>
-    <row r="19" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:80">
       <c r="A19" s="4" t="s">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="B19" s="5">
         <v>2.5629465996438476</v>
@@ -18269,9 +18333,9 @@
         <v>2.0449992152373242</v>
       </c>
     </row>
-    <row r="20" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:80">
       <c r="A20" s="4" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="B20" s="5">
         <v>2.3223223223223184</v>
@@ -18511,9 +18575,9 @@
         <v>3.0335533315456695</v>
       </c>
     </row>
-    <row r="21" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:80">
       <c r="A21" s="4" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="B21" s="5">
         <v>0.86161656842285705</v>
@@ -18753,9 +18817,9 @@
         <v>1.6145216550202905</v>
       </c>
     </row>
-    <row r="22" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:80">
       <c r="A22" s="4" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="B22" s="5">
         <v>4.1216250832522281</v>
@@ -18995,9 +19059,9 @@
         <v>2.9313370626302495</v>
       </c>
     </row>
-    <row r="23" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:80">
       <c r="A23" s="4" t="s">
-        <v>19</v>
+        <v>103</v>
       </c>
       <c r="B23" s="5">
         <v>3.87880578695547</v>
@@ -19237,9 +19301,9 @@
         <v>1.4816179373141358</v>
       </c>
     </row>
-    <row r="24" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:80">
       <c r="A24" s="4" t="s">
-        <v>20</v>
+        <v>104</v>
       </c>
       <c r="B24" s="5">
         <v>-0.47730866919058174</v>
@@ -19479,9 +19543,9 @@
         <v>1.3366525167894465</v>
       </c>
     </row>
-    <row r="25" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:80">
       <c r="A25" s="4" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="B25" s="5">
         <v>1.2648516170280732</v>
@@ -19721,9 +19785,9 @@
         <v>1.0584151285391721</v>
       </c>
     </row>
-    <row r="26" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:80">
       <c r="A26" s="4" t="s">
-        <v>22</v>
+        <v>106</v>
       </c>
       <c r="B26" s="5">
         <v>2.78260652067884</v>
@@ -19963,9 +20027,9 @@
         <v>0.98268815723009506</v>
       </c>
     </row>
-    <row r="27" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:80">
       <c r="A27" s="4" t="s">
-        <v>23</v>
+        <v>107</v>
       </c>
       <c r="B27" s="5">
         <v>2.5086848953325709</v>
@@ -20205,9 +20269,9 @@
         <v>2.4083769633507957</v>
       </c>
     </row>
-    <row r="28" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:80">
       <c r="A28" s="4" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="B28" s="5">
         <v>-2.0222519095646563</v>
@@ -20447,9 +20511,9 @@
         <v>1.8408652335861273</v>
       </c>
     </row>
-    <row r="29" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:80">
       <c r="A29" s="4" t="s">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="B29" s="5">
         <v>1.2317896482293038</v>
@@ -20689,9 +20753,9 @@
         <v>1.2204363610729274</v>
       </c>
     </row>
-    <row r="30" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:80">
       <c r="A30" s="4" t="s">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="B30" s="5">
         <v>1.9187358916478654</v>
@@ -20931,9 +20995,9 @@
         <v>1.530951852673619</v>
       </c>
     </row>
-    <row r="31" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:80">
       <c r="A31" s="4" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="B31" s="5">
         <v>1.2012441064304289</v>
@@ -21173,9 +21237,9 @@
         <v>1.6324954360342658</v>
       </c>
     </row>
-    <row r="32" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:80">
       <c r="A32" s="4" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
       <c r="B32" s="5">
         <v>1.3634320531388922</v>
@@ -21415,9 +21479,9 @@
         <v>2.5493178723031544</v>
       </c>
     </row>
-    <row r="33" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:80">
       <c r="A33" s="4" t="s">
-        <v>29</v>
+        <v>113</v>
       </c>
       <c r="B33" s="5">
         <v>3.3114518829563782</v>
@@ -21657,9 +21721,9 @@
         <v>2.2384088338987511</v>
       </c>
     </row>
-    <row r="34" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:80">
       <c r="A34" s="4" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="B34" s="5">
         <v>4.9322439218812253</v>
@@ -21899,9 +21963,9 @@
         <v>2.1144385949771163</v>
       </c>
     </row>
-    <row r="35" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:80">
       <c r="A35" s="4" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="B35" s="5">
         <v>2.0743271099593801</v>
@@ -22141,9 +22205,9 @@
         <v>2.6342988442910724</v>
       </c>
     </row>
-    <row r="36" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:80">
       <c r="A36" s="4" t="s">
-        <v>32</v>
+        <v>116</v>
       </c>
       <c r="B36" s="5">
         <v>1.9058736254145667</v>
@@ -22383,9 +22447,9 @@
         <v>2.0178903952245806</v>
       </c>
     </row>
-    <row r="37" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:80">
       <c r="A37" s="4" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="B37" s="5">
         <v>1.5490293036355347</v>
@@ -22625,9 +22689,9 @@
         <v>1.7304267348986333</v>
       </c>
     </row>
-    <row r="38" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:80">
       <c r="A38" s="4" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="B38" s="5">
         <v>5.4065061345008418</v>
@@ -22867,9 +22931,9 @@
         <v>3.0207081648583864</v>
       </c>
     </row>
-    <row r="39" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:80">
       <c r="A39" s="4" t="s">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="B39" s="5">
         <v>6.2477513801873394</v>
@@ -23109,9 +23173,9 @@
         <v>3.0150465805458642</v>
       </c>
     </row>
-    <row r="40" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:80">
       <c r="A40" s="4" t="s">
-        <v>36</v>
+        <v>120</v>
       </c>
       <c r="B40" s="5">
         <v>2.376910016977944</v>
@@ -23351,9 +23415,9 @@
         <v>0.67443231558073102</v>
       </c>
     </row>
-    <row r="41" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:80">
       <c r="A41" s="4" t="s">
-        <v>37</v>
+        <v>121</v>
       </c>
       <c r="B41" s="5">
         <v>0.50668464217502218</v>
@@ -23593,9 +23657,9 @@
         <v>2.1630376102213442</v>
       </c>
     </row>
-    <row r="42" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:80">
       <c r="A42" s="4" t="s">
-        <v>38</v>
+        <v>122</v>
       </c>
       <c r="B42" s="5">
         <v>10.222723583387216</v>
@@ -23835,9 +23899,9 @@
         <v>1.6947300361530135</v>
       </c>
     </row>
-    <row r="43" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:80">
       <c r="A43" s="4" t="s">
-        <v>39</v>
+        <v>123</v>
       </c>
       <c r="B43" s="5">
         <v>5.7471419691359671</v>
@@ -24077,9 +24141,9 @@
         <v>1.0987327551723811</v>
       </c>
     </row>
-    <row r="44" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:80">
       <c r="A44" s="4" t="s">
-        <v>40</v>
+        <v>124</v>
       </c>
       <c r="B44" s="5">
         <v>0.11551977820203586</v>
@@ -24319,9 +24383,9 @@
         <v>2.3421436315376321</v>
       </c>
     </row>
-    <row r="45" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:80">
       <c r="A45" s="4" t="s">
-        <v>41</v>
+        <v>125</v>
       </c>
       <c r="B45" s="5">
         <v>2.1211797392605241</v>
@@ -24561,9 +24625,9 @@
         <v>1.3516505821785108</v>
       </c>
     </row>
-    <row r="46" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:80">
       <c r="A46" s="4" t="s">
-        <v>42</v>
+        <v>126</v>
       </c>
       <c r="B46" s="5">
         <v>2.6031118794764074</v>
@@ -24803,9 +24867,9 @@
         <v>3.5288142152278419</v>
       </c>
     </row>
-    <row r="47" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:80">
       <c r="A47" s="4" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="B47" s="5">
         <v>1.066533895862271</v>
@@ -25045,9 +25109,9 @@
         <v>2.2565533025784088</v>
       </c>
     </row>
-    <row r="48" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:80">
       <c r="A48" s="4" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="B48" s="5">
         <v>2.6784051258490371</v>
@@ -25287,9 +25351,9 @@
         <v>2.1239236060999755</v>
       </c>
     </row>
-    <row r="49" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:80">
       <c r="A49" s="4" t="s">
-        <v>45</v>
+        <v>129</v>
       </c>
       <c r="B49" s="5">
         <v>4.6811545683468907</v>
@@ -25529,9 +25593,9 @@
         <v>2.4901206361491774</v>
       </c>
     </row>
-    <row r="50" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:80">
       <c r="A50" s="4" t="s">
-        <v>46</v>
+        <v>130</v>
       </c>
       <c r="B50" s="5">
         <v>7.7133715306198596</v>
@@ -25771,9 +25835,9 @@
         <v>3.0268000204859633</v>
       </c>
     </row>
-    <row r="51" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:80">
       <c r="A51" s="4" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="B51" s="5">
         <v>1.4593901555270714</v>
@@ -26013,9 +26077,9 @@
         <v>1.540323370024641</v>
       </c>
     </row>
-    <row r="52" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:80">
       <c r="A52" s="4" t="s">
-        <v>48</v>
+        <v>132</v>
       </c>
       <c r="B52" s="5">
         <v>3.6677938846453957</v>
@@ -26255,9 +26319,9 @@
         <v>2.1359759619006056</v>
       </c>
     </row>
-    <row r="53" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:80">
       <c r="A53" s="4" t="s">
-        <v>49</v>
+        <v>133</v>
       </c>
       <c r="B53" s="5">
         <v>4.1782190024744441</v>
@@ -26497,9 +26561,9 @@
         <v>2.2939410684150032</v>
       </c>
     </row>
-    <row r="54" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:80">
       <c r="A54" s="4" t="s">
-        <v>50</v>
+        <v>134</v>
       </c>
       <c r="B54" s="5">
         <v>1.6169417211025972</v>
@@ -26739,9 +26803,9 @@
         <v>1.6903922693698541</v>
       </c>
     </row>
-    <row r="55" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:80">
       <c r="A55" s="4" t="s">
-        <v>51</v>
+        <v>135</v>
       </c>
       <c r="B55" s="5">
         <v>2.2551375967432477</v>
@@ -26981,9 +27045,9 @@
         <v>1.5446105542373127</v>
       </c>
     </row>
-    <row r="56" spans="1:80" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:80">
       <c r="A56" s="4" t="s">
-        <v>52</v>
+        <v>136</v>
       </c>
       <c r="B56" s="5">
         <v>6.7681816600368707</v>

</xml_diff>